<commit_message>
Optimize bandwidth for Render
</commit_message>
<xml_diff>
--- a/Uploader_Config.xlsx
+++ b/Uploader_Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\NEET Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670BA023-0E6B-4E47-A575-46B78D368A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEE3AFFF-1CA5-41C0-B5C3-45103E8934B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SR ELITE" sheetId="3" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="8">
   <si>
     <t>STUD_ID</t>
   </si>
@@ -87,7 +87,68 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -424,13 +485,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9782594E-49BA-43C6-9E7A-F1DB7B294A92}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.625" customWidth="1"/>
     <col min="2" max="2" width="21.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -438,7 +499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>246400791</v>
       </c>
@@ -446,7 +507,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>246400986</v>
       </c>
@@ -918,14 +979,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B81"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B112"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.625" customWidth="1"/>
     <col min="2" max="2" width="21.625" customWidth="1"/>
+    <col min="7" max="7" width="12.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -933,17 +995,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>257403546</v>
+        <v>246556443</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>246556034</v>
+        <v>246556442</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -951,7 +1013,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>246556345</v>
+        <v>246556441</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
@@ -959,7 +1021,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>246562584</v>
+        <v>246556444</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
@@ -967,7 +1029,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>213307618</v>
+        <v>257403546</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -975,7 +1037,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>257403520</v>
+        <v>257404738</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
@@ -983,7 +1045,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>213309261</v>
+        <v>257403653</v>
       </c>
       <c r="B8" t="s">
         <v>2</v>
@@ -991,7 +1053,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>246556008</v>
+        <v>213309261</v>
       </c>
       <c r="B9" t="s">
         <v>2</v>
@@ -999,7 +1061,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>257409613</v>
+        <v>246556034</v>
       </c>
       <c r="B10" t="s">
         <v>2</v>
@@ -1007,7 +1069,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>257404738</v>
+        <v>246556008</v>
       </c>
       <c r="B11" t="s">
         <v>2</v>
@@ -1015,7 +1077,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>257418223</v>
+        <v>224308526</v>
       </c>
       <c r="B12" t="s">
         <v>2</v>
@@ -1023,7 +1085,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>246556423</v>
+        <v>246556786</v>
       </c>
       <c r="B13" t="s">
         <v>2</v>
@@ -1031,7 +1093,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>246556436</v>
+        <v>213307618</v>
       </c>
       <c r="B14" t="s">
         <v>2</v>
@@ -1039,7 +1101,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>257402548</v>
+        <v>246556423</v>
       </c>
       <c r="B15" t="s">
         <v>2</v>
@@ -1047,7 +1109,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>257405184</v>
+        <v>257403856</v>
       </c>
       <c r="B16" t="s">
         <v>2</v>
@@ -1055,7 +1117,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>213309273</v>
+        <v>246562584</v>
       </c>
       <c r="B17" t="s">
         <v>2</v>
@@ -1063,7 +1125,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>257401230</v>
+        <v>257427698</v>
       </c>
       <c r="B18" t="s">
         <v>2</v>
@@ -1071,7 +1133,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>257414545</v>
+        <v>257403520</v>
       </c>
       <c r="B19" t="s">
         <v>2</v>
@@ -1079,7 +1141,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>246556409</v>
+        <v>224308589</v>
       </c>
       <c r="B20" t="s">
         <v>2</v>
@@ -1087,7 +1149,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>246556664</v>
+        <v>246556799</v>
       </c>
       <c r="B21" t="s">
         <v>2</v>
@@ -1095,7 +1157,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>246556443</v>
+        <v>257409613</v>
       </c>
       <c r="B22" t="s">
         <v>2</v>
@@ -1103,7 +1165,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>257402253</v>
+        <v>257405184</v>
       </c>
       <c r="B23" t="s">
         <v>2</v>
@@ -1111,7 +1173,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>246556442</v>
+        <v>257405810</v>
       </c>
       <c r="B24" t="s">
         <v>2</v>
@@ -1119,7 +1181,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>246556441</v>
+        <v>257414545</v>
       </c>
       <c r="B25" t="s">
         <v>2</v>
@@ -1127,7 +1189,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>246556444</v>
+        <v>257403566</v>
       </c>
       <c r="B26" t="s">
         <v>2</v>
@@ -1135,255 +1197,255 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>246555726</v>
+        <v>246556345</v>
       </c>
       <c r="B27" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>257409631</v>
+        <v>246555884</v>
       </c>
       <c r="B28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>257400127</v>
+        <v>246556409</v>
       </c>
       <c r="B29" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>246555676</v>
+        <v>213307653</v>
       </c>
       <c r="B30" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>257403841</v>
+        <v>246556664</v>
       </c>
       <c r="B31" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>257403863</v>
+        <v>257425334</v>
       </c>
       <c r="B32" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>257403517</v>
+        <v>257403537</v>
       </c>
       <c r="B33" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>257404572</v>
+        <v>213309273</v>
       </c>
       <c r="B34" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>257403831</v>
+        <v>257407693</v>
       </c>
       <c r="B35" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>257419001</v>
+        <v>257405813</v>
       </c>
       <c r="B36" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>257406595</v>
+        <v>257428306</v>
       </c>
       <c r="B37" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>246555720</v>
+        <v>235419458</v>
       </c>
       <c r="B38" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>246555684</v>
+        <v>246556811</v>
       </c>
       <c r="B39" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>257405190</v>
+        <v>257402253</v>
       </c>
       <c r="B40" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>257407126</v>
+        <v>257407705</v>
       </c>
       <c r="B41" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>257404775</v>
+        <v>246556668</v>
       </c>
       <c r="B42" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>257404510</v>
+        <v>246556436</v>
       </c>
       <c r="B43" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>246569203</v>
+        <v>257405229</v>
       </c>
       <c r="B44" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>257405746</v>
+        <v>257400521</v>
       </c>
       <c r="B45" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>257403867</v>
+        <v>213309192</v>
       </c>
       <c r="B46" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>257409625</v>
+        <v>257403536</v>
       </c>
       <c r="B47" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>257404573</v>
+        <v>257418223</v>
       </c>
       <c r="B48" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>257418337</v>
+        <v>257402548</v>
       </c>
       <c r="B49" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>257406437</v>
+        <v>246556019</v>
       </c>
       <c r="B50" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>246555700</v>
+        <v>257403555</v>
       </c>
       <c r="B51" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>257407741</v>
+        <v>257401230</v>
       </c>
       <c r="B52" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>257406414</v>
+        <v>213309257</v>
       </c>
       <c r="B53" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>257407096</v>
+        <v>257405203</v>
       </c>
       <c r="B54" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>246555705</v>
+        <v>246556007</v>
       </c>
       <c r="B55" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>257407748</v>
+        <v>257405219</v>
       </c>
       <c r="B56" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>257409620</v>
+        <v>257420307</v>
       </c>
       <c r="B57" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>257422296</v>
+        <v>246555726</v>
       </c>
       <c r="B58" t="s">
         <v>3</v>
@@ -1391,7 +1453,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>257406447</v>
+        <v>257409631</v>
       </c>
       <c r="B59" t="s">
         <v>3</v>
@@ -1399,7 +1461,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>257409786</v>
+        <v>257400127</v>
       </c>
       <c r="B60" t="s">
         <v>3</v>
@@ -1407,7 +1469,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>257403382</v>
+        <v>246555676</v>
       </c>
       <c r="B61" t="s">
         <v>3</v>
@@ -1415,7 +1477,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>257380023</v>
+        <v>257403841</v>
       </c>
       <c r="B62" t="s">
         <v>3</v>
@@ -1423,7 +1485,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>257405159</v>
+        <v>257403863</v>
       </c>
       <c r="B63" t="s">
         <v>3</v>
@@ -1431,7 +1493,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>246555713</v>
+        <v>257403517</v>
       </c>
       <c r="B64" t="s">
         <v>3</v>
@@ -1439,7 +1501,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>257403873</v>
+        <v>257404572</v>
       </c>
       <c r="B65" t="s">
         <v>3</v>
@@ -1447,7 +1509,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>257417304</v>
+        <v>257403831</v>
       </c>
       <c r="B66" t="s">
         <v>3</v>
@@ -1455,7 +1517,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>257404516</v>
+        <v>257419001</v>
       </c>
       <c r="B67" t="s">
         <v>3</v>
@@ -1463,7 +1525,7 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>257407133</v>
+        <v>257406595</v>
       </c>
       <c r="B68" t="s">
         <v>3</v>
@@ -1471,7 +1533,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>257405195</v>
+        <v>246555720</v>
       </c>
       <c r="B69" t="s">
         <v>3</v>
@@ -1479,7 +1541,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>257406421</v>
+        <v>246555684</v>
       </c>
       <c r="B70" t="s">
         <v>3</v>
@@ -1487,7 +1549,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>257410225</v>
+        <v>257405190</v>
       </c>
       <c r="B71" t="s">
         <v>3</v>
@@ -1495,7 +1557,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>257407134</v>
+        <v>257407126</v>
       </c>
       <c r="B72" t="s">
         <v>3</v>
@@ -1503,7 +1565,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>257406448</v>
+        <v>257404775</v>
       </c>
       <c r="B73" t="s">
         <v>3</v>
@@ -1511,7 +1573,7 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>257428648</v>
+        <v>257404510</v>
       </c>
       <c r="B74" t="s">
         <v>3</v>
@@ -1519,7 +1581,7 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>257404564</v>
+        <v>246569203</v>
       </c>
       <c r="B75" t="s">
         <v>3</v>
@@ -1527,7 +1589,7 @@
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>257403819</v>
+        <v>257405746</v>
       </c>
       <c r="B76" t="s">
         <v>3</v>
@@ -1535,7 +1597,7 @@
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>257405854</v>
+        <v>257403867</v>
       </c>
       <c r="B77" t="s">
         <v>3</v>
@@ -1543,7 +1605,7 @@
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>257403851</v>
+        <v>257409625</v>
       </c>
       <c r="B78" t="s">
         <v>3</v>
@@ -1551,7 +1613,7 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>257407906</v>
+        <v>257404573</v>
       </c>
       <c r="B79" t="s">
         <v>3</v>
@@ -1559,7 +1621,7 @@
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>257417639</v>
+        <v>257418337</v>
       </c>
       <c r="B80" t="s">
         <v>3</v>
@@ -1567,16 +1629,273 @@
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81">
+        <v>257406437</v>
+      </c>
+      <c r="B81" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>246555700</v>
+      </c>
+      <c r="B82" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>257407741</v>
+      </c>
+      <c r="B83" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>257406414</v>
+      </c>
+      <c r="B84" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>257407096</v>
+      </c>
+      <c r="B85" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>246555705</v>
+      </c>
+      <c r="B86" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>257407748</v>
+      </c>
+      <c r="B87" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>257409620</v>
+      </c>
+      <c r="B88" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>257422296</v>
+      </c>
+      <c r="B89" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>257406447</v>
+      </c>
+      <c r="B90" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>257409786</v>
+      </c>
+      <c r="B91" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>257403382</v>
+      </c>
+      <c r="B92" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>257380023</v>
+      </c>
+      <c r="B93" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>257405159</v>
+      </c>
+      <c r="B94" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>246555713</v>
+      </c>
+      <c r="B95" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>257403873</v>
+      </c>
+      <c r="B96" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>257417304</v>
+      </c>
+      <c r="B97" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>257404516</v>
+      </c>
+      <c r="B98" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>257407133</v>
+      </c>
+      <c r="B99" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>257405195</v>
+      </c>
+      <c r="B100" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>257406421</v>
+      </c>
+      <c r="B101" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>257410225</v>
+      </c>
+      <c r="B102" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>257407134</v>
+      </c>
+      <c r="B103" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>257406448</v>
+      </c>
+      <c r="B104" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>257428648</v>
+      </c>
+      <c r="B105" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>257404564</v>
+      </c>
+      <c r="B106" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>257403819</v>
+      </c>
+      <c r="B107" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>257405854</v>
+      </c>
+      <c r="B108" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>257403851</v>
+      </c>
+      <c r="B109" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>257407906</v>
+      </c>
+      <c r="B110" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>257417639</v>
+      </c>
+      <c r="B111" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112">
         <v>257426969</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B112" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:A57 A113:A1048576">
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B113:B141">
+    <cfRule type="duplicateValues" dxfId="3" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:B1 B2" numberStoredAsText="1"/>
+    <ignoredError sqref="B1 B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1585,19 +1904,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>

</xml_diff>